<commit_message>
ElyTable kept results: array members by cell (booleans, empty strings, bad numbers), ODS empty strings in any attribute order and without a paragraph (R14.37 round 2)
</commit_message>
<xml_diff>
--- a/tests/fixtures/table/kept-more.xlsx
+++ b/tests/fixtures/table/kept-more.xlsx
@@ -30,6 +30,10 @@
       <c r="E1">
         <f t="array" ref="E1">CUBEVALUE("Sales","[Measures].[Total]")</f>
         <v>41</v>
+      </c>
+      <c r="J1" t="b">
+        <f t="array" ref="J1">FUTUREFN(9)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="2">
@@ -82,6 +86,60 @@
         <v>43</v>
       </c>
     </row>
+    <row r="10">
+      <c r="G10" t="b">
+        <f t="array" ref="G10:H10">FUTUREFN(5)</f>
+        <v>1</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="G11">
+        <f t="array" ref="G11:H11">FUTUREFN(6)</f>
+        <v>41</v>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="G12">
+        <f t="array" ref="G12:H12">FUTUREFN(7)</f>
+        <v>41</v>
+      </c>
+      <c r="H12">
+        <v>not-a-number</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="G13">
+        <f t="array" ref="G13:H13">FUTUREFN(8)</f>
+        <v>41</v>
+      </c>
+      <c r="H13">
+        <v>42garbage</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="G14" t="b">
+        <f t="array" ref="G14:H14">FUTUREFN(10)</f>
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="G15">
+        <f t="array" ref="G15:H15">FUTUREFN(11)</f>
+        <v>41</v>
+      </c>
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>